<commit_message>
NETCARB NIVAL v1.1 validée, AZUR v1.2 : polluants revus
NIVAL portait une courbe empruntée à AZUR, des mentions de travail et
une photo provisoire. Passe de contenu faite avec Pierre-Alain, sur la
base d'AZUR :
- sous-titre « Filtre caisson multidièdre à charbon actif », descriptif
  et points clés rédigés par PA, caractéristiques alignées sur AZUR ;
- pas de courbe tant que celle du NIVAL n'est pas mesurée : nouvelle clé
  opt-in sans_courbe (fiche sur une page, sans colonne ΔP, catalogue
  sans graphique et caractéristiques remontées) ;
- photo Netair à cadre noir, codes NETCARB-NIVAL-CA-….

AZUR v1.2 et NIVAL : le badge et la ligne Fonction disent « gaz, odeurs
et COV » au lieu de « COV · O₃ · SO₂ · NO₂ ». Ces quatre gaz sont ceux
de l'essai ISO 10121-3 et aucune mesure ne les soutient.

Registre, DONNEES_PDC, catalogue, site, CHECKLIST et PROCESS à jour.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fiches-techniques/Bibliotheque_Fiches_Techniques_Netair.xlsx
+++ b/fiches-techniques/Bibliotheque_Fiches_Techniques_Netair.xlsx
@@ -1517,7 +1517,7 @@
       </c>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>v1.1</t>
+          <t>v1.2</t>
         </is>
       </c>
       <c r="H18" s="6" t="inlineStr">
@@ -1527,7 +1527,7 @@
       </c>
       <c r="I18" s="8" t="inlineStr">
         <is>
-          <t>Validée PA — contenu retravaillé 12/10 (sous-titre, descriptif et points clés PA, courbe 2023 à 122 Pa, photo Netair, codes CA)</t>
+          <t>Validée PA — contenu retravaillé 12/10 (sous-titre, descriptif et points clés PA, courbe 2023 à 122 Pa, photo Netair, codes CA) ; v1.2 12/10 : ligne Fonction et badge : « gaz, odeurs et COV » au lieu des 4 gaz non mesurés (accord PA)</t>
         </is>
       </c>
       <c r="J18" s="7" t="inlineStr">
@@ -1564,7 +1564,7 @@
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>Polydièdre charbon actif</t>
+          <t>Filtre caisson multidièdre, charbon actif</t>
         </is>
       </c>
       <c r="E19" s="6" t="inlineStr">
@@ -1574,22 +1574,22 @@
       </c>
       <c r="F19" s="6" t="inlineStr">
         <is>
-          <t>Moléculaire (ISO 10121)</t>
+          <t>Moléculaire (aucune classe ISO 10121 affichée)</t>
         </is>
       </c>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>v1.0</t>
+          <t>v1.1</t>
         </is>
       </c>
       <c r="H19" s="6" t="inlineStr">
         <is>
-          <t>23/06/2026</t>
+          <t>12/10/2026</t>
         </is>
       </c>
       <c r="I19" s="8" t="inlineStr">
         <is>
-          <t>Créée — charbon actif polydièdre, mono-classe 292 mm (courbe partagée AZUR)</t>
+          <t>Validée PA — contenu retravaillé 12/10 (sous-titre, descriptif et points clés PA, photo Netair cadre noir, sans courbe : fiche 1 page, polluants « gaz, odeurs et COV », codes CA)</t>
         </is>
       </c>
       <c r="J19" s="7" t="inlineStr">
@@ -1604,7 +1604,7 @@
       </c>
       <c r="L19" s="7" t="inlineStr">
         <is>
-          <t>Polydièdre charbon (gaz). ⚠ Aucune courbe ΔP V-CARB mesurée → courbe pack charbon 292 mm de SV-GD/QL partagée (à mesurer R&amp;D). Nominal 3000, ΔP@3000≈80. Combinable F7. T° 40°C, HR 70%, feu NA. Parois polyester à confirmer. Photo Q-carb (code visible→remplacer). Classe LD/MD/HD &amp; capacité→R&amp;D.</t>
+          <t>v1.1 12/10/2026, décisions PA : base NETCARB AZUR v1.1. Sous-titre « Filtre caisson multidièdre à charbon actif » ; descriptif et points clés PA ; même média qu'AZUR (grains entre deux médias non tissés) ; capacité sans chiffre ; parois « Plastique » ; aucune mention ISO 10121 ; polluants « gaz, odeurs et COV » (badge + Fonction) au lieu des 4 gaz non mesurés. PAS DE COURBE pour le moment (clé sans_courbe) : aucune mesure du V-CARB charbon seul ; la fiche V-CARB F7 2018 (combinée) recopie QL-CARB F9 2013, l'ancienne courbe empruntée (QL-CARB 2013) est abandonnée. Débits 3 000 / 2 480 / 1 450. Codes NETCARB-NIVAL-CA-LxHxP. Donnée non affichée : masse de charbon 2 748 g (V-CARB F7 2018).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
NETCARB BAG v1.1 validée : données du fournisseur, photo Netair
La fiche décrivait un F9 en poches de 520 mm d'après une fiche Titanair,
avec des mentions de travail et la photo du NETBAG S. Les données
techniques suivent désormais la fiche du fournisseur réel :
- ePM1 50 % (F7), fibres de verre et grains de charbon actif ;
- 9 formats (592, 490, 287 × 592 ; poches de 635, 535, 380 mm), avec
  la surface de média et la ΔP du fournisseur par référence ;
- pas de courbe (un seul point par profondeur) : fiche sur une page ;
- codes NETCARB-BAG-F7CA-…, sous-titre, descriptif et points clés de PA.

Générateur : deux réglages opt-in, dims_dp_tableau (ΔP par ligne sans
courbe) et surface par ligne ; les 17 autres fiches sont inchangées.
Configurateur : formats standard (largeur + profondeur) et sur mesure.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fiches-techniques/Bibliotheque_Fiches_Techniques_Netair.xlsx
+++ b/fiches-techniques/Bibliotheque_Fiches_Techniques_Netair.xlsx
@@ -1626,32 +1626,32 @@
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>Poches charbon actif</t>
+          <t>Filtre à poches souples, particules + charbon actif</t>
         </is>
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>F9</t>
+          <t>F7</t>
         </is>
       </c>
       <c r="F20" s="6" t="inlineStr">
         <is>
-          <t>ePM1 80% + CA (ISO 10121)</t>
+          <t>ePM1 50% (équivalence table, non mesurée)</t>
         </is>
       </c>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>v1.0</t>
+          <t>v1.1</t>
         </is>
       </c>
       <c r="H20" s="6" t="inlineStr">
         <is>
-          <t>23/06/2026</t>
+          <t>12/10/2026</t>
         </is>
       </c>
       <c r="I20" s="8" t="inlineStr">
         <is>
-          <t>Créée — poches souples F9 à charbon imprégné (combiné), mono-classe 520</t>
+          <t>Validée PA — contenu retravaillé 12/10 (données techniques fournisseur F7, 9 formats, ΔP par profondeur sans courbe, textes PA, photo Netair, codes F7CA)</t>
         </is>
       </c>
       <c r="J20" s="7" t="inlineStr">
@@ -1661,12 +1661,12 @@
       </c>
       <c r="K20" s="6" t="inlineStr">
         <is>
-          <t>TITABAG F9 CARB</t>
+          <t>Deltricarb GCA (fournisseur) ; v1.0 : TITABAG F9 CA</t>
         </is>
       </c>
       <c r="L20" s="7" t="inlineStr">
         <is>
-          <t>COMBINÉ particules+charbon (≠ charbon grains) : classe ISO 16890 F9 ePM1 80% PRIMAIRE + charbon imprégné (odeurs/COV, capacité 15%). COLMATANT → règle ePM +100 (pas const). 9,172·v²+64,135·v−10,429 ; ΔP@3400≈229. Cadre acier, 520mm, T° 40°C, feu NA. HR n.c. Photo forme poches NETBAG placeholder (média imprégné à reshooter).</t>
+          <t>v1.1 12/10/2026, décisions PA : données techniques reprises de la fiche fournisseur Deltricarb GCA (BLOC3/Fournisseurs/DELTRIAN) au lieu de TITABAG F9 CA 2021. Classe EN 779 F7 → ePM1 50 % (F7) par la table de correspondance ; média fibres de verre + grains de charbon actif ; profondeurs 635/535/380 ; formats 592/490/287×592 ; surfaces de média par référence ; ΔP fournisseur 105/130/145 Pa par profondeur (pas de courbe : clés sans_courbe + dims_dp_tableau) ; T° affichée 40 °C max. comme AZUR/NIVAL (source : 50 °C continu) ; HR 70 % ; cadre acier galvanisé et feu « Non classé » ajoutés par PA (absents de la source). Non repris : ΔP finale 450 Pa (règle gamme +100), contact alimentaire CE 1935/2004 (sans certificat). Capacité sans chiffre. Codes NETCARB-BAG-F7CA-LxHxP. Sur-mesure confirmé par PA. Photo Netair « Netcarb Bag.png ». ΔP finale : « Charbon saturé ou poches colmatées (ΔP initiale + 100 Pa) ».</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
NETCARB CILIA v1.1 validée : famille NETCARB terminée
CILIA affichait des mentions de travail, la photo de grains de
charbon, et deux défauts : la courbe 98 mm était étiquetée « 48 mm » au
catalogue, et la ligne 98 mm du tableau portait la ΔP du 48 (73 au lieu
de 67 Pa). Passe de contenu faite avec Pierre-Alain :
- sous-titre, descriptif et points clés de PA, photo Netair ;
- tableau aligné sur AZUR et NIVAL (média, gaz, odeurs et COV, capacité
  sans chiffre, Non classé, 40 °C max.) ; cadre acier galvanisé ou
  cellulose pelliculée, HR 50 % et épaisseurs 48 / 98 mm restent sourcés ;
- codes NETCARB-CILIA-CA-…, courbe tracée en débit jusqu'à 4 000 m³/h.

Générateur : en mode deux épaisseurs, chaque ligne prend la ΔP de son
épaisseur (seule CILIA concernée). Configurateur : efficacité figée
« Charbon actif » (le prix s'affiche d'emblée), cadre au choix -A / -C.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fiches-techniques/Bibliotheque_Fiches_Techniques_Netair.xlsx
+++ b/fiches-techniques/Bibliotheque_Fiches_Techniques_Netair.xlsx
@@ -1440,7 +1440,7 @@
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>Compact charbon actif</t>
+          <t>Filtre compact miniplis, charbon actif</t>
         </is>
       </c>
       <c r="E17" s="6" t="inlineStr">
@@ -1450,22 +1450,22 @@
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
-          <t>Moléculaire (ISO 10121)</t>
+          <t>Moléculaire (aucune classe ISO 10121 affichée)</t>
         </is>
       </c>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>v1.0</t>
+          <t>v1.1</t>
         </is>
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t>23/06/2026</t>
+          <t>12/10/2026</t>
         </is>
       </c>
       <c r="I17" s="8" t="inlineStr">
         <is>
-          <t>Créée — filtre moléculaire charbon actif, 2 épaisseurs 48/98 mm</t>
+          <t>Validée PA — contenu retravaillé 12/10 (sous-titre, descriptif et points clés PA, photo Netair, alignement famille, épaisseurs 48/98 corrigées, codes CA)</t>
         </is>
       </c>
       <c r="J17" s="7" t="inlineStr">
@@ -1480,7 +1480,7 @@
       </c>
       <c r="L17" s="7" t="inlineStr">
         <is>
-          <t>Charbon actif pur (gaz) : pas de classe ePM. ISO 10121 (LD/MD/HD à déterminer). ΔP réelles caches Excel 48/98 (cohérentes 48&gt;98), poly 7 pts. ΔP non colmatante (remplacement à saturation, capacité 15% masse). T° 40°C, HR 50%, feu NA. Nouveaux drapeaux moteur deux_epaisseurs + dp_final_mode:const. Photo CARB.png (grains) placeholder.</t>
+          <t>v1.1 12/10/2026, décisions PA : sous-titre « Filtre compact charbon actif » ; descriptif et points clés PA ; média libellé comme AZUR (sources : micro-grains) ; capacité sans chiffre (sources : 15 %) ; polluants « gaz, odeurs et COV » ; feu « Non classé » ; 40 °C max. ; HR 50 % (doc 2015) ; cadre acier galvanisé ou cellulose pelliculée ; toutes dimensions comme NETPAK S CILIA. Corrections : étiquette d'épaisseur (la courbe 98 était nommée 48 au catalogue), ligne 98 mm du tableau 73 → 67 Pa (moteur). Courbes PRISME CARB 48/98 inchangées (73/67 Pa @3400). Codes NETCARB-CILIA-CA-LxHxP. Photo « Netcarb Cilia.png ». Configurateur : efficacité figée « Charbon actif » (prix affiché d'emblée), cadre au choix -A/-C.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
NETPAK S CILIA DUO v1.1 validée : les 18 fiches ont eu leur passe
L'ancien « NETPAK S DUO » ne décrivait qu'un F7 + charbon, avec des
codes article cassés, deux valeurs sans source et une photo de compact
simple. Passe de contenu faite avec Pierre-Alain :
- renommé NETPAK S CILIA DUO partout (fiche, site, catalogue,
  configurateur), comme le prévoit la codification ;
- DUO = deux packs miniplis dans un cadre : particules + particules ou
  particules + charbon ; plage M5 → F9 annoncée, courbe et calculateur
  de la version ePM1 50 % (F7) + charbon (190 Pa à 3 400 m³/h) ;
- textes et photo de PA, cadre acier galvanisé ou cellulose pelliculée,
  feu M1 / non classé ; surface 12,6 m² et HR 100 % retirées (sans source).

Générateur : clé opt-in ref_base (code NETPAK-CILIA-DUO-F7CA-…).
Configurateur : deux menus d'efficacité (M5 → F9 et charbon), sans
doublon, charbon toujours en fin de code ; cadre au choix.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fiches-techniques/Bibliotheque_Fiches_Techniques_Netair.xlsx
+++ b/fiches-techniques/Bibliotheque_Fiches_Techniques_Netair.xlsx
@@ -1673,12 +1673,12 @@
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>FT-NETPAK-S-DUO</t>
+          <t>FT-NETPAK-S-CILIA-DUO</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>NETPAK S DUO</t>
+          <t>NETPAK S CILIA DUO</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
@@ -1688,37 +1688,37 @@
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>Compact mini-plis + charbon actif</t>
+          <t>Compact miniplis double filtration (2 packs)</t>
         </is>
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>F7 + CA</t>
+          <t>M5 → F9</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr">
         <is>
-          <t>ePM1 50% + CA</t>
+          <t>ePM10 50% → ePM1 80% (+ charbon actif)</t>
         </is>
       </c>
       <c r="G21" s="6" t="inlineStr">
         <is>
-          <t>v1.0</t>
+          <t>v1.1</t>
         </is>
       </c>
       <c r="H21" s="6" t="inlineStr">
         <is>
-          <t>22/06/2026</t>
+          <t>12/10/2026</t>
         </is>
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
-          <t>Créée — mono-classe F7 GREENTEX + charbon actif (ep48)</t>
+          <t>Validée PA — contenu retravaillé 12/10 (renommé NETPAK S CILIA DUO, 2 packs miniplis, plage M5 → F9, courbe ePM1 50 % (F7) + charbon, textes et photo PA)</t>
         </is>
       </c>
       <c r="J21" s="7" t="inlineStr">
         <is>
-          <t>Fiches_Netair/Fiche technique NETPAK S DUO.html</t>
+          <t>Fiches_Netair/Fiche technique NETPAK S CILIA DUO.html</t>
         </is>
       </c>
       <c r="K21" s="6" t="inlineStr">
@@ -1728,7 +1728,7 @@
       </c>
       <c r="L21" s="7" t="inlineStr">
         <is>
-          <t>F7 GREENTEX + charbon actif. ΔP combinée 36→247 Pa (nom 190). Feu NA (charbon non classé). Surface média dév. ≈12,55 m². ΔP finale +100 Pa (= règle Titanair PDC init+100). Photo placeholder PRISME A à remplacer. Capacité CA (grammage) non communiquée → R&amp;D. MAJ 17/07/2026 : libellé humidité passé à « 100 % (sans condensation) » (déc. PA). ⚠️ VERSION VOLONTAIREMENT NON BUMPÉE (reste v1.0) : la passe de contenu de cette fiche n'a pas eu lieu, bumper en v1.1 consommerait le numéro qu'elle mérite. Décision PA du 17/07. La fiche affiche donc « v1.0 — 22/06/2026 » alors que sa ligne humidité date du 17/07 — écart connu et assumé.</t>
+          <t>v1.1 12/10/2026, décisions PA : renommé NETPAK S CILIA DUO partout (ex-NETPAK S DUO, slug netpak-s-cilia-duo) ; DUO = 2 packs miniplis dans un cadre, particules + particules (ex. M5F7) ou particules + charbon (F7CA) ; plage M5 → F9 annoncée (modèle BORA) ; courbe et calculateur ePM1 50 % (F7) + charbon 48 mm (source DUO F7 GR-CA ep48 du 10/10/2022 : 36…247 Pa, 190 Pa @3400) ; 60 °C (65 °C / 1 h) ; feu M1 (particulaire) / non classé (charbon) ; cadre acier galvanisé ou cellulose pelliculée (CODIFICATION_PRODUITS.md mise à jour) ; capacité sans chiffre. Retirés car non sourcés : surface 12,6 m², HR 100 %. Codes NETPAK-CILIA-DUO-F7CA-LxHxP (clé ref_base). Configurateur : sur devis, Efficacité 1 et 2 (M5 → F9 + charbon, sans doublon, CA en fin de code), cadre au choix. Titre 26 px pour tenir sur une ligne. Photo Netair en écorché.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
NETCEL V NIVAL v1.2 validée : « caisson multidièdre »
Le filtre absolu NIVAL a la même forme de caisson que le NETCARB NIVAL,
mais sa fiche disait « polydièdre » et son sous-titre ne nommait pas la
forme. Sous-titre « Filtre absolu caisson multidièdre », même mot dans
le descriptif et la ligne Type, badge « Filtre absolu (T.H.E) » au lieu
de « Polydièdre ». Fiche passée en v1.2, validée par Pierre-Alain.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fiches-techniques/Bibliotheque_Fiches_Techniques_Netair.xlsx
+++ b/fiches-techniques/Bibliotheque_Fiches_Techniques_Netair.xlsx
@@ -1316,7 +1316,7 @@
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>Filtre polydièdre T.H.E</t>
+          <t>Filtre absolu caisson multidièdre</t>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr">
@@ -1331,17 +1331,17 @@
       </c>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>v1.1</t>
+          <t>v1.2</t>
         </is>
       </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>15/08/2026</t>
+          <t>12/10/2026</t>
         </is>
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
-          <t>Contenu retravaillé v1.1 — courbes E10 + H13 réelles, 4 formats, cadre 610×610 corrigé (H14 à mesurer)</t>
+          <t>Validée PA — contenu retravaillé v1.1 (15/08) ; v1.2 (12/10) : « caisson multidièdre » (sous-titre, descriptif, Type), badge « Filtre absolu (T.H.E) »</t>
         </is>
       </c>
       <c r="J15" s="7" t="inlineStr">

</xml_diff>

<commit_message>
Registre : NETCEL V AZUR validée, les 18 fiches sont validées
NETCEL V AZUR (v1.2 du 15/08) était retravaillée mais jamais marquée
validée : Pierre-Alain la valide telle quelle. Les points laissés
ouverts (forme polydièdre / multidièdre, mentions sans source,
température) sont notés à la CHECKLIST. NETFIL : la mention « photo à
remplacer » du registre était périmée depuis le 22/09.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fiches-techniques/Bibliotheque_Fiches_Techniques_Netair.xlsx
+++ b/fiches-techniques/Bibliotheque_Fiches_Techniques_Netair.xlsx
@@ -721,7 +721,7 @@
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
-          <t>Validée PA — contenu retravaillé (photo à remplacer)</t>
+          <t>Validée PA — contenu retravaillé (photo Netair depuis le 22/09)</t>
         </is>
       </c>
       <c r="J5" s="7" t="inlineStr">
@@ -1279,7 +1279,7 @@
       </c>
       <c r="I14" s="8" t="inlineStr">
         <is>
-          <t>Contenu retravaillé v1.1 (02/08) — v1.2 (15/08) : ligne « Séparateur : Hot melt » ajoutée (accord PA)</t>
+          <t>Validée PA (12/10/2026, sans retouche) — contenu retravaillé v1.1 (02/08), v1.2 (15/08)</t>
         </is>
       </c>
       <c r="J14" s="7" t="inlineStr">

</xml_diff>

<commit_message>
NETBAG S v1.2 : la fiche tient de nouveau sur 2 pages à l'impression
À l'impression, NETBAG S sortait sur 4 pages : la page 1 dépassait de
6,4 mm, la page 2 de 21 mm (défaut antérieur, déjà présent sur main).
Mise en page seule, aucun contenu changé, avec l'accord de Pierre-Alain :
- specs_serre : lignes du tableau des caractéristiques à 4 px ;
- calc_serre : interligne des curseurs du calculateur 7 px, marges −1 mm ;
- courbe à 70 % de largeur au lieu de 85 %.
Marges restantes mesurées : page 1 6,3 mm, page 2 2,9 mm. Les deux
réglages sont opt-in : les 17 autres fiches ne bougent pas.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fiches-techniques/Bibliotheque_Fiches_Techniques_Netair.xlsx
+++ b/fiches-techniques/Bibliotheque_Fiches_Techniques_Netair.xlsx
@@ -959,17 +959,17 @@
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>v1.1</t>
+          <t>v1.2</t>
         </is>
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>26/07/2026</t>
+          <t>12/10/2026</t>
         </is>
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
-          <t>Validée PA — contenu retravaillé 26/07 (densité progressive, stock F7 par défaut, courbe/curseur bornés 4 000, boutique code 17 : standard 380/550 chiffrés, G4/M5 et sur-mesure en devis)</t>
+          <t>Validée PA — contenu retravaillé 26/07 (densité progressive, stock F7 par défaut, courbe/curseur bornés 4 000, boutique code 17 : standard 380/550 chiffrés, G4/M5 et sur-mesure en devis) ; v1.2 12/10 : mise en page corrigée, la fiche sortait sur 4 pages à l'impression (accord PA)</t>
         </is>
       </c>
       <c r="J9" s="7" t="inlineStr">

</xml_diff>

<commit_message>
NETBAG S v1.3 : la mesure douteuse du M5 550 mm est retirée
La donnée source du M5 en poches de 550 mm (49 Pa à 3 400 m³/h) est plus
basse que celle du 650 mm (65 Pa) alors qu'il a moins de média :
physiquement incohérent, sans doute deux étiquettes interverties. Elle
s'affichait avec « (à valider) » et « valeur à confirmer », dernières
mentions de travail visibles de la gamme. Sur décision de Pierre-Alain,
courbe et ligne sont retirées jusqu'à une mesure ; les données restent
dans le JSON (_m5_550_retire) et le M5 550 mm reste vendable sur devis.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fiches-techniques/Bibliotheque_Fiches_Techniques_Netair.xlsx
+++ b/fiches-techniques/Bibliotheque_Fiches_Techniques_Netair.xlsx
@@ -959,7 +959,7 @@
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>v1.2</t>
+          <t>v1.3</t>
         </is>
       </c>
       <c r="H9" s="6" t="inlineStr">
@@ -969,7 +969,7 @@
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
-          <t>Validée PA — contenu retravaillé 26/07 (densité progressive, stock F7 par défaut, courbe/curseur bornés 4 000, boutique code 17 : standard 380/550 chiffrés, G4/M5 et sur-mesure en devis) ; v1.2 12/10 : mise en page corrigée, la fiche sortait sur 4 pages à l'impression (accord PA)</t>
+          <t>Validée PA — contenu retravaillé 26/07 (densité progressive, stock F7 par défaut, courbe/curseur bornés 4 000, boutique code 17 : standard 380/550 chiffrés, G4/M5 et sur-mesure en devis) ; v1.2 12/10 : mise en page corrigée, la fiche sortait sur 4 pages à l'impression (accord PA) ; v1.3 12/10 : courbe et ligne M5 550 mm retirées (mesure incohérente, à mesurer), plus aucune mention « à valider » (accord PA)</t>
         </is>
       </c>
       <c r="J9" s="7" t="inlineStr">

</xml_diff>

<commit_message>
Badges de gamme alignés sur les produits réels (audit, accord PA)
Préfiltres : Coarse 40 % → ePM10 50 % (G2 → M5) au lieu de Coarse 65 % (G3 → M5) ;
miniplis : à partir de G4 (NETPAK S BORA) ; absolus : E10 → U15 (NETCEL V LAM).
NETPLAN : badge Coarse 40 % → 65 % (G2 → G4) comme sa fiche et son configurateur,
fiche v1.3 (seul diff : badges et version), registre à jour.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fiches-techniques/Bibliotheque_Fiches_Techniques_Netair.xlsx
+++ b/fiches-techniques/Bibliotheque_Fiches_Techniques_Netair.xlsx
@@ -897,17 +897,17 @@
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>v1.2</t>
+          <t>v1.3</t>
         </is>
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>17/07/2026</t>
+          <t>12/10/2026</t>
         </is>
       </c>
       <c r="I8" s="8" t="inlineStr">
         <is>
-          <t>Validée PA — contenu retravaillé 16/07</t>
+          <t>Validée PA — contenu retravaillé 16/07 ; v1.3 (12/10) : badges alignés sur la gamme réelle « Coarse 40 % → 65 % (G2 → G4) » au lieu de « Coarse 65 % (G4) » (audit, accord PA)</t>
         </is>
       </c>
       <c r="J8" s="7" t="inlineStr">

</xml_diff>